<commit_message>
Final sync, formatting fixes, exe build, ready for PR
</commit_message>
<xml_diff>
--- a/company_data.xlsx
+++ b/company_data.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="661" uniqueCount="291">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="600" uniqueCount="289">
   <si>
     <t xml:space="preserve">Type</t>
   </si>
@@ -710,22 +710,16 @@
     <t xml:space="preserve">EFT</t>
   </si>
   <si>
-    <t xml:space="preserve">23-0375</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Test2</t>
-  </si>
-  <si>
     <t xml:space="preserve">23-0401</t>
   </si>
   <si>
     <t xml:space="preserve">NBT Group LTD</t>
   </si>
   <si>
-    <t xml:space="preserve">.......</t>
-  </si>
-  <si>
-    <t xml:space="preserve">23-0402</t>
+    <t xml:space="preserve">EX-500</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ExcelOnly</t>
   </si>
   <si>
     <t xml:space="preserve">5054</t>
@@ -995,7 +989,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1046,6 +1040,10 @@
     </xf>
     <xf numFmtId="170" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -1101,16 +1099,16 @@
         <a:srgbClr val="467886"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Sheets">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Arial" pitchFamily="0" charset="1"/>
-        <a:ea typeface="Arial" pitchFamily="0" charset="1"/>
-        <a:cs typeface="Arial" pitchFamily="0" charset="1"/>
+        <a:ea typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+        <a:cs typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Arial" pitchFamily="0" charset="1"/>
-        <a:ea typeface="Arial" pitchFamily="0" charset="1"/>
-        <a:cs typeface="Arial" pitchFamily="0" charset="1"/>
+        <a:ea typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+        <a:cs typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme>
@@ -1118,67 +1116,25 @@
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:gradFill>
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:lumMod val="110000"/>
-                <a:tint val="67000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="50000">
-              <a:schemeClr val="phClr">
-                <a:lumMod val="105000"/>
-                <a:tint val="73000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:lumMod val="105000"/>
-                <a:tint val="81000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
-        </a:gradFill>
-        <a:gradFill>
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:lumMod val="102000"/>
-                <a:tint val="94000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="50000">
-              <a:schemeClr val="phClr">
-                <a:lumMod val="100000"/>
-                <a:shade val="100000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:lumMod val="99000"/>
-                <a:shade val="78000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
-        </a:gradFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
         <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
+          <a:miter/>
         </a:ln>
-        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
+          <a:miter/>
         </a:ln>
-        <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
+          <a:miter/>
         </a:ln>
       </a:lnStyleLst>
       <a:effectStyleLst>
@@ -1197,35 +1153,11 @@
           <a:schemeClr val="phClr"/>
         </a:solidFill>
         <a:solidFill>
-          <a:schemeClr val="phClr">
-            <a:tint val="95000"/>
-          </a:schemeClr>
+          <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:gradFill>
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:tint val="93000"/>
-                <a:shade val="98000"/>
-                <a:lumMod val="102000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="50000">
-              <a:schemeClr val="phClr">
-                <a:tint val="98000"/>
-                <a:shade val="90000"/>
-                <a:lumMod val="103000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:shade val="63000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
-        </a:gradFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
@@ -9328,11 +9260,16 @@
   <dimension ref="A1:Z1000"/>
   <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="1" style="1" width="11.38"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="1" width="11.38"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="18.28"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="1" width="11.38"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="18.18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="7" style="1" width="11.38"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="13.75"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="10" style="1" width="11.38"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="26.73"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="24.6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="9" style="1" width="18.22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="11" style="1" width="11.38"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="19.8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="1" width="11.38"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="26" min="16" style="1" width="8.63"/>
   </cols>
   <sheetData>
@@ -9396,10 +9333,10 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="9" t="n">
-        <v>4931</v>
+        <v>4950</v>
       </c>
       <c r="B2" s="9" t="n">
-        <v>7502</v>
+        <v>7535</v>
       </c>
       <c r="C2" s="9" t="s">
         <v>224</v>
@@ -9408,10 +9345,10 @@
         <v>45126</v>
       </c>
       <c r="E2" s="11" t="n">
-        <v>45408</v>
+        <v>45422</v>
       </c>
       <c r="F2" s="12" t="n">
-        <v>1882.26</v>
+        <v>946.11</v>
       </c>
       <c r="G2" s="9" t="n">
         <v>47900</v>
@@ -9420,7 +9357,7 @@
         <v>117</v>
       </c>
       <c r="I2" s="12" t="n">
-        <v>8475.15</v>
+        <v>0</v>
       </c>
       <c r="J2" s="9" t="s">
         <v>225</v>
@@ -9435,7 +9372,7 @@
         <v>182</v>
       </c>
       <c r="N2" s="12" t="n">
-        <v>1882.26</v>
+        <v>946.11</v>
       </c>
       <c r="O2" s="10"/>
       <c r="P2" s="10"/>
@@ -9452,22 +9389,22 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="9" t="n">
-        <v>4927</v>
+        <v>5008</v>
       </c>
       <c r="B3" s="9" t="n">
-        <v>7498</v>
+        <v>7656</v>
       </c>
       <c r="C3" s="9" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
       <c r="D3" s="11" t="n">
-        <v>45126</v>
+        <v>45182</v>
       </c>
       <c r="E3" s="11" t="n">
-        <v>45401</v>
+        <v>45485</v>
       </c>
       <c r="F3" s="12" t="n">
-        <v>1903.11</v>
+        <v>2162.35</v>
       </c>
       <c r="G3" s="9" t="n">
         <v>47900</v>
@@ -9476,10 +9413,10 @@
         <v>117</v>
       </c>
       <c r="I3" s="12" t="n">
-        <v>8475.15</v>
+        <v>13100</v>
       </c>
       <c r="J3" s="9" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
       <c r="K3" s="9" t="s">
         <v>226</v>
@@ -9491,7 +9428,7 @@
         <v>182</v>
       </c>
       <c r="N3" s="12" t="n">
-        <v>1903.11</v>
+        <v>2162.35</v>
       </c>
       <c r="O3" s="10"/>
       <c r="P3" s="10"/>
@@ -9507,23 +9444,23 @@
       <c r="Z3" s="10"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="9" t="n">
-        <v>4950</v>
-      </c>
-      <c r="B4" s="9" t="n">
-        <v>7535</v>
-      </c>
-      <c r="C4" s="9" t="s">
-        <v>224</v>
-      </c>
-      <c r="D4" s="11" t="n">
-        <v>45126</v>
+      <c r="A4" s="1" t="n">
+        <v>5050</v>
+      </c>
+      <c r="B4" s="1" t="n">
+        <v>5000</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>229</v>
+      </c>
+      <c r="D4" s="13" t="n">
+        <v>44941</v>
       </c>
       <c r="E4" s="11" t="n">
-        <v>45422</v>
+        <v>45546</v>
       </c>
       <c r="F4" s="12" t="n">
-        <v>946.11</v>
+        <v>400</v>
       </c>
       <c r="G4" s="9" t="n">
         <v>47900</v>
@@ -9532,10 +9469,10 @@
         <v>117</v>
       </c>
       <c r="I4" s="12" t="n">
-        <v>8475.15</v>
-      </c>
-      <c r="J4" s="9" t="s">
-        <v>225</v>
+        <v>5040</v>
+      </c>
+      <c r="J4" s="1" t="s">
+        <v>230</v>
       </c>
       <c r="K4" s="9" t="s">
         <v>226</v>
@@ -9547,64 +9484,24 @@
         <v>182</v>
       </c>
       <c r="N4" s="12" t="n">
-        <v>946.11</v>
-      </c>
-      <c r="O4" s="10"/>
-      <c r="P4" s="10"/>
-      <c r="Q4" s="10"/>
-      <c r="R4" s="10"/>
-      <c r="S4" s="10"/>
-      <c r="T4" s="10"/>
-      <c r="U4" s="10"/>
-      <c r="V4" s="10"/>
-      <c r="W4" s="10"/>
-      <c r="X4" s="10"/>
-      <c r="Y4" s="10"/>
-      <c r="Z4" s="10"/>
+        <v>2162.35</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="9" t="n">
-        <v>4911</v>
-      </c>
-      <c r="B5" s="9" t="n">
-        <v>7473</v>
-      </c>
-      <c r="C5" s="9" t="s">
-        <v>224</v>
-      </c>
-      <c r="D5" s="11" t="n">
-        <v>45126</v>
-      </c>
-      <c r="E5" s="11" t="n">
-        <v>45394</v>
-      </c>
-      <c r="F5" s="12" t="n">
-        <v>1861.41</v>
-      </c>
-      <c r="G5" s="9" t="n">
-        <v>47900</v>
-      </c>
-      <c r="H5" s="9" t="s">
-        <v>117</v>
-      </c>
-      <c r="I5" s="12" t="n">
-        <v>8475.15</v>
-      </c>
-      <c r="J5" s="9" t="s">
-        <v>225</v>
-      </c>
-      <c r="K5" s="9" t="s">
-        <v>226</v>
-      </c>
-      <c r="L5" s="9" t="s">
-        <v>115</v>
-      </c>
-      <c r="M5" s="9" t="s">
-        <v>182</v>
-      </c>
-      <c r="N5" s="12" t="n">
-        <v>1861.41</v>
-      </c>
+      <c r="A5" s="9"/>
+      <c r="B5" s="9"/>
+      <c r="C5" s="9"/>
+      <c r="D5" s="11"/>
+      <c r="E5" s="11"/>
+      <c r="F5" s="12"/>
+      <c r="G5" s="9"/>
+      <c r="H5" s="9"/>
+      <c r="I5" s="12"/>
+      <c r="J5" s="9"/>
+      <c r="K5" s="9"/>
+      <c r="L5" s="9"/>
+      <c r="M5" s="9"/>
+      <c r="N5" s="12"/>
       <c r="O5" s="10"/>
       <c r="P5" s="10"/>
       <c r="Q5" s="10"/>
@@ -9618,105 +9515,21 @@
       <c r="Y5" s="10"/>
       <c r="Z5" s="10"/>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="9" t="n">
-        <v>4945</v>
-      </c>
-      <c r="B6" s="9" t="n">
-        <v>7529</v>
-      </c>
-      <c r="C6" s="9" t="s">
-        <v>224</v>
-      </c>
-      <c r="D6" s="11" t="n">
-        <v>45126</v>
-      </c>
-      <c r="E6" s="11" t="n">
-        <v>45415</v>
-      </c>
-      <c r="F6" s="12" t="n">
-        <v>1882.26</v>
-      </c>
-      <c r="G6" s="9" t="n">
-        <v>47900</v>
-      </c>
-      <c r="H6" s="9" t="s">
-        <v>117</v>
-      </c>
-      <c r="I6" s="12" t="n">
-        <v>8475.15</v>
-      </c>
-      <c r="J6" s="9" t="s">
-        <v>225</v>
-      </c>
-      <c r="K6" s="9" t="s">
-        <v>226</v>
-      </c>
-      <c r="L6" s="9" t="s">
-        <v>115</v>
-      </c>
-      <c r="M6" s="9" t="s">
-        <v>182</v>
-      </c>
-      <c r="N6" s="12" t="n">
-        <v>1882.26</v>
-      </c>
-      <c r="O6" s="10"/>
-      <c r="P6" s="10"/>
-      <c r="Q6" s="10"/>
-      <c r="R6" s="10"/>
-      <c r="S6" s="10"/>
-      <c r="T6" s="10"/>
-      <c r="U6" s="10"/>
-      <c r="V6" s="10"/>
-      <c r="W6" s="10"/>
-      <c r="X6" s="10"/>
-      <c r="Y6" s="10"/>
-      <c r="Z6" s="10"/>
-    </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="9" t="n">
-        <v>4859</v>
-      </c>
-      <c r="B7" s="9" t="n">
-        <v>7377</v>
-      </c>
-      <c r="C7" s="9" t="s">
-        <v>227</v>
-      </c>
-      <c r="D7" s="11" t="n">
-        <v>45176</v>
-      </c>
-      <c r="E7" s="11" t="n">
-        <v>45323</v>
-      </c>
-      <c r="F7" s="12" t="n">
-        <v>4256</v>
-      </c>
-      <c r="G7" s="9" t="n">
-        <v>47900</v>
-      </c>
-      <c r="H7" s="9" t="s">
-        <v>117</v>
-      </c>
-      <c r="I7" s="12" t="n">
-        <v>4256</v>
-      </c>
-      <c r="J7" s="9" t="s">
-        <v>228</v>
-      </c>
-      <c r="K7" s="9" t="s">
-        <v>226</v>
-      </c>
-      <c r="L7" s="9" t="s">
-        <v>115</v>
-      </c>
-      <c r="M7" s="9" t="s">
-        <v>182</v>
-      </c>
-      <c r="N7" s="12" t="n">
-        <v>4256</v>
-      </c>
+      <c r="A7" s="9"/>
+      <c r="B7" s="9"/>
+      <c r="C7" s="9"/>
+      <c r="D7" s="11"/>
+      <c r="E7" s="11"/>
+      <c r="F7" s="12"/>
+      <c r="G7" s="9"/>
+      <c r="H7" s="9"/>
+      <c r="I7" s="12"/>
+      <c r="J7" s="9"/>
+      <c r="K7" s="9"/>
+      <c r="L7" s="9"/>
+      <c r="M7" s="9"/>
+      <c r="N7" s="12"/>
       <c r="O7" s="10"/>
       <c r="P7" s="10"/>
       <c r="Q7" s="10"/>
@@ -9731,51 +9544,21 @@
       <c r="Z7" s="10"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="9" t="n">
-        <v>4959</v>
-      </c>
-      <c r="B8" s="9" t="n">
-        <v>7548</v>
-      </c>
-      <c r="C8" s="9" t="s">
-        <v>229</v>
-      </c>
-      <c r="D8" s="11" t="n">
-        <v>45182</v>
-      </c>
-      <c r="E8" s="11" t="n">
-        <v>45436</v>
-      </c>
-      <c r="F8" s="12" t="n">
-        <v>1882.26</v>
-      </c>
-      <c r="G8" s="9" t="n">
-        <v>47900</v>
-      </c>
-      <c r="H8" s="9" t="s">
-        <v>117</v>
-      </c>
-      <c r="I8" s="12" t="n">
-        <v>13100</v>
-      </c>
-      <c r="J8" s="9" t="s">
-        <v>230</v>
-      </c>
-      <c r="K8" s="9" t="s">
-        <v>226</v>
-      </c>
-      <c r="L8" s="9" t="s">
-        <v>115</v>
-      </c>
-      <c r="M8" s="9" t="s">
-        <v>182</v>
-      </c>
-      <c r="N8" s="12" t="n">
-        <v>1882.26</v>
-      </c>
-      <c r="O8" s="12" t="n">
-        <v>1040.98</v>
-      </c>
+      <c r="A8" s="9"/>
+      <c r="B8" s="9"/>
+      <c r="C8" s="9"/>
+      <c r="D8" s="11"/>
+      <c r="E8" s="11"/>
+      <c r="F8" s="12"/>
+      <c r="G8" s="9"/>
+      <c r="H8" s="9"/>
+      <c r="I8" s="12"/>
+      <c r="J8" s="9"/>
+      <c r="K8" s="9"/>
+      <c r="L8" s="9"/>
+      <c r="M8" s="9"/>
+      <c r="N8" s="12"/>
+      <c r="O8" s="12"/>
       <c r="P8" s="10"/>
       <c r="Q8" s="10"/>
       <c r="R8" s="10"/>
@@ -9788,105 +9571,21 @@
       <c r="Y8" s="10"/>
       <c r="Z8" s="10"/>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="9" t="n">
-        <v>5008</v>
-      </c>
-      <c r="B9" s="9" t="n">
-        <v>7656</v>
-      </c>
-      <c r="C9" s="9" t="s">
-        <v>229</v>
-      </c>
-      <c r="D9" s="11" t="n">
-        <v>45182</v>
-      </c>
-      <c r="E9" s="11" t="n">
-        <v>45485</v>
-      </c>
-      <c r="F9" s="12" t="n">
-        <v>2162.35</v>
-      </c>
-      <c r="G9" s="9" t="n">
-        <v>47900</v>
-      </c>
-      <c r="H9" s="9" t="s">
-        <v>117</v>
-      </c>
-      <c r="I9" s="12" t="n">
-        <v>13100</v>
-      </c>
-      <c r="J9" s="9" t="s">
-        <v>230</v>
-      </c>
-      <c r="K9" s="9" t="s">
-        <v>226</v>
-      </c>
-      <c r="L9" s="9" t="s">
-        <v>115</v>
-      </c>
-      <c r="M9" s="9" t="s">
-        <v>182</v>
-      </c>
-      <c r="N9" s="12" t="n">
-        <v>2162.35</v>
-      </c>
-      <c r="O9" s="10"/>
-      <c r="P9" s="10"/>
-      <c r="Q9" s="10"/>
-      <c r="R9" s="10"/>
-      <c r="S9" s="10"/>
-      <c r="T9" s="10"/>
-      <c r="U9" s="10"/>
-      <c r="V9" s="10"/>
-      <c r="W9" s="10"/>
-      <c r="X9" s="10"/>
-      <c r="Y9" s="10"/>
-      <c r="Z9" s="10"/>
-    </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="9" t="n">
-        <v>4956</v>
-      </c>
-      <c r="B10" s="9" t="n">
-        <v>7544</v>
-      </c>
-      <c r="C10" s="9" t="s">
-        <v>229</v>
-      </c>
-      <c r="D10" s="11" t="n">
-        <v>45182</v>
-      </c>
-      <c r="E10" s="11" t="n">
-        <v>45429</v>
-      </c>
-      <c r="F10" s="12" t="n">
-        <v>1882.26</v>
-      </c>
-      <c r="G10" s="9" t="n">
-        <v>47900</v>
-      </c>
-      <c r="H10" s="9" t="s">
-        <v>117</v>
-      </c>
-      <c r="I10" s="12" t="n">
-        <v>13100</v>
-      </c>
-      <c r="J10" s="9" t="s">
-        <v>230</v>
-      </c>
-      <c r="K10" s="9" t="s">
-        <v>226</v>
-      </c>
-      <c r="L10" s="9" t="s">
-        <v>115</v>
-      </c>
-      <c r="M10" s="9" t="s">
-        <v>182</v>
-      </c>
-      <c r="N10" s="12" t="n">
-        <v>1882.26</v>
-      </c>
+      <c r="A10" s="9"/>
+      <c r="B10" s="9"/>
+      <c r="C10" s="9"/>
+      <c r="D10" s="11"/>
+      <c r="E10" s="11"/>
+      <c r="F10" s="12"/>
+      <c r="G10" s="9"/>
+      <c r="H10" s="9"/>
+      <c r="I10" s="12"/>
+      <c r="J10" s="9"/>
+      <c r="K10" s="9"/>
+      <c r="L10" s="9"/>
+      <c r="M10" s="9"/>
+      <c r="N10" s="12"/>
       <c r="O10" s="10"/>
       <c r="P10" s="10"/>
       <c r="Q10" s="10"/>
@@ -9901,48 +9600,20 @@
       <c r="Z10" s="10"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="9" t="s">
-        <v>231</v>
-      </c>
-      <c r="B11" s="9" t="n">
-        <v>7648</v>
-      </c>
-      <c r="C11" s="9" t="s">
-        <v>229</v>
-      </c>
-      <c r="D11" s="11" t="n">
-        <v>45182</v>
-      </c>
-      <c r="E11" s="11" t="n">
-        <v>45476</v>
-      </c>
-      <c r="F11" s="12" t="n">
-        <v>1732</v>
-      </c>
-      <c r="G11" s="9" t="n">
-        <v>47900</v>
-      </c>
-      <c r="H11" s="9" t="s">
-        <v>117</v>
-      </c>
-      <c r="I11" s="12" t="n">
-        <v>13100</v>
-      </c>
-      <c r="J11" s="9" t="s">
-        <v>230</v>
-      </c>
-      <c r="K11" s="9" t="s">
-        <v>226</v>
-      </c>
-      <c r="L11" s="9" t="s">
-        <v>115</v>
-      </c>
-      <c r="M11" s="9" t="s">
-        <v>182</v>
-      </c>
-      <c r="N11" s="12" t="n">
-        <v>1732</v>
-      </c>
+      <c r="A11" s="9"/>
+      <c r="B11" s="9"/>
+      <c r="C11" s="9"/>
+      <c r="D11" s="11"/>
+      <c r="E11" s="11"/>
+      <c r="F11" s="12"/>
+      <c r="G11" s="9"/>
+      <c r="H11" s="9"/>
+      <c r="I11" s="12"/>
+      <c r="J11" s="9"/>
+      <c r="K11" s="9"/>
+      <c r="L11" s="9"/>
+      <c r="M11" s="9"/>
+      <c r="N11" s="12"/>
       <c r="O11" s="10"/>
       <c r="P11" s="10"/>
       <c r="Q11" s="10"/>
@@ -9957,48 +9628,20 @@
       <c r="Z11" s="10"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="9" t="n">
-        <v>4950</v>
-      </c>
-      <c r="B12" s="9" t="n">
-        <v>7536</v>
-      </c>
-      <c r="C12" s="9" t="s">
-        <v>229</v>
-      </c>
-      <c r="D12" s="11" t="n">
-        <v>45182</v>
-      </c>
-      <c r="E12" s="11" t="n">
-        <v>45422</v>
-      </c>
-      <c r="F12" s="12" t="n">
-        <v>936.15</v>
-      </c>
-      <c r="G12" s="9" t="n">
-        <v>47900</v>
-      </c>
-      <c r="H12" s="9" t="s">
-        <v>117</v>
-      </c>
-      <c r="I12" s="12" t="n">
-        <v>13100</v>
-      </c>
-      <c r="J12" s="9" t="s">
-        <v>230</v>
-      </c>
-      <c r="K12" s="9" t="s">
-        <v>226</v>
-      </c>
-      <c r="L12" s="9" t="s">
-        <v>115</v>
-      </c>
-      <c r="M12" s="9" t="s">
-        <v>182</v>
-      </c>
-      <c r="N12" s="12" t="n">
-        <v>936.15</v>
-      </c>
+      <c r="A12" s="9"/>
+      <c r="B12" s="9"/>
+      <c r="C12" s="9"/>
+      <c r="D12" s="11"/>
+      <c r="E12" s="11"/>
+      <c r="F12" s="12"/>
+      <c r="G12" s="9"/>
+      <c r="H12" s="9"/>
+      <c r="I12" s="12"/>
+      <c r="J12" s="9"/>
+      <c r="K12" s="9"/>
+      <c r="L12" s="9"/>
+      <c r="M12" s="9"/>
+      <c r="N12" s="12"/>
       <c r="O12" s="10"/>
       <c r="P12" s="10"/>
       <c r="Q12" s="10"/>
@@ -10013,48 +9656,20 @@
       <c r="Z12" s="10"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="9" t="n">
-        <v>4994</v>
-      </c>
-      <c r="B13" s="9" t="n">
-        <v>7626</v>
-      </c>
-      <c r="C13" s="9" t="s">
-        <v>229</v>
-      </c>
-      <c r="D13" s="11" t="n">
-        <v>45182</v>
-      </c>
-      <c r="E13" s="11" t="n">
-        <v>45471</v>
-      </c>
-      <c r="F13" s="12" t="n">
-        <v>1732</v>
-      </c>
-      <c r="G13" s="9" t="n">
-        <v>47900</v>
-      </c>
-      <c r="H13" s="9" t="s">
-        <v>117</v>
-      </c>
-      <c r="I13" s="12" t="n">
-        <v>13100</v>
-      </c>
-      <c r="J13" s="9" t="s">
-        <v>230</v>
-      </c>
-      <c r="K13" s="9" t="s">
-        <v>226</v>
-      </c>
-      <c r="L13" s="9" t="s">
-        <v>115</v>
-      </c>
-      <c r="M13" s="9" t="s">
-        <v>182</v>
-      </c>
-      <c r="N13" s="12" t="n">
-        <v>1732</v>
-      </c>
+      <c r="A13" s="9"/>
+      <c r="B13" s="9"/>
+      <c r="C13" s="9"/>
+      <c r="D13" s="11"/>
+      <c r="E13" s="11"/>
+      <c r="F13" s="12"/>
+      <c r="G13" s="9"/>
+      <c r="H13" s="9"/>
+      <c r="I13" s="12"/>
+      <c r="J13" s="9"/>
+      <c r="K13" s="9"/>
+      <c r="L13" s="9"/>
+      <c r="M13" s="9"/>
+      <c r="N13" s="12"/>
       <c r="O13" s="10"/>
       <c r="P13" s="10"/>
       <c r="Q13" s="10"/>
@@ -10069,48 +9684,20 @@
       <c r="Z13" s="10"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="9" t="n">
-        <v>5029</v>
-      </c>
-      <c r="B14" s="9" t="n">
-        <v>7688</v>
-      </c>
-      <c r="C14" s="9" t="s">
-        <v>232</v>
-      </c>
-      <c r="D14" s="11" t="n">
-        <v>45182</v>
-      </c>
-      <c r="E14" s="11" t="n">
-        <v>45499</v>
-      </c>
-      <c r="F14" s="12" t="n">
-        <v>1732</v>
-      </c>
-      <c r="G14" s="9" t="n">
-        <v>47900</v>
-      </c>
-      <c r="H14" s="9" t="s">
-        <v>117</v>
-      </c>
-      <c r="I14" s="12" t="n">
-        <v>13100</v>
-      </c>
-      <c r="J14" s="9" t="s">
-        <v>230</v>
-      </c>
-      <c r="K14" s="9" t="s">
-        <v>226</v>
-      </c>
-      <c r="L14" s="9" t="s">
-        <v>115</v>
-      </c>
-      <c r="M14" s="9" t="s">
-        <v>182</v>
-      </c>
-      <c r="N14" s="12" t="n">
-        <v>1732</v>
-      </c>
+      <c r="A14" s="9"/>
+      <c r="B14" s="9"/>
+      <c r="C14" s="9"/>
+      <c r="D14" s="11"/>
+      <c r="E14" s="11"/>
+      <c r="F14" s="12"/>
+      <c r="G14" s="9"/>
+      <c r="H14" s="9"/>
+      <c r="I14" s="12"/>
+      <c r="J14" s="9"/>
+      <c r="K14" s="9"/>
+      <c r="L14" s="9"/>
+      <c r="M14" s="9"/>
+      <c r="N14" s="12"/>
       <c r="O14" s="10"/>
       <c r="P14" s="10"/>
       <c r="Q14" s="10"/>
@@ -10184,7 +9771,7 @@
       <c r="M17" s="5"/>
       <c r="N17" s="8"/>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="21" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="22" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="23" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
@@ -11242,10 +10829,10 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="C2" s="7"/>
       <c r="D2" s="8"/>
@@ -11263,7 +10850,7 @@
         <v>34</v>
       </c>
       <c r="J2" s="5" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="K2" s="5" t="s">
         <v>179</v>
@@ -11281,10 +10868,10 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="5" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="C3" s="7"/>
       <c r="D3" s="8"/>
@@ -11302,7 +10889,7 @@
         <v>34</v>
       </c>
       <c r="J3" s="5" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="K3" s="5" t="s">
         <v>179</v>
@@ -11320,10 +10907,10 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="C4" s="7"/>
       <c r="D4" s="8"/>
@@ -11341,7 +10928,7 @@
         <v>34</v>
       </c>
       <c r="J4" s="5" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="K4" s="5" t="s">
         <v>179</v>
@@ -11359,10 +10946,10 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="C5" s="7"/>
       <c r="D5" s="8"/>
@@ -11398,10 +10985,10 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="C6" s="7"/>
       <c r="D6" s="8"/>
@@ -11419,7 +11006,7 @@
         <v>77</v>
       </c>
       <c r="J6" s="5" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="K6" s="5" t="s">
         <v>179</v>
@@ -11437,10 +11024,10 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="C7" s="7"/>
       <c r="D7" s="8"/>
@@ -11458,7 +11045,7 @@
         <v>129</v>
       </c>
       <c r="J7" s="5" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="K7" s="5"/>
       <c r="L7" s="5" t="s">
@@ -11474,10 +11061,10 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="C8" s="7"/>
       <c r="D8" s="8"/>
@@ -11495,7 +11082,7 @@
         <v>129</v>
       </c>
       <c r="J8" s="5" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="K8" s="5"/>
       <c r="L8" s="5" t="s">
@@ -11511,10 +11098,10 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="C9" s="7"/>
       <c r="D9" s="8"/>
@@ -11532,7 +11119,7 @@
         <v>129</v>
       </c>
       <c r="J9" s="5" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="K9" s="5"/>
       <c r="L9" s="5" t="s">
@@ -11548,10 +11135,10 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="C10" s="7"/>
       <c r="D10" s="8"/>
@@ -11569,7 +11156,7 @@
         <v>129</v>
       </c>
       <c r="J10" s="5" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="K10" s="5"/>
       <c r="L10" s="5" t="s">
@@ -11585,10 +11172,10 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="C11" s="7"/>
       <c r="D11" s="8"/>
@@ -11606,7 +11193,7 @@
         <v>129</v>
       </c>
       <c r="J11" s="5" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="K11" s="5"/>
       <c r="L11" s="5" t="s">
@@ -11622,10 +11209,10 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="5" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="C12" s="7"/>
       <c r="D12" s="8"/>
@@ -11643,7 +11230,7 @@
         <v>129</v>
       </c>
       <c r="J12" s="5" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="K12" s="5"/>
       <c r="L12" s="5" t="s">
@@ -11659,10 +11246,10 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="5" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="C13" s="7"/>
       <c r="D13" s="8"/>
@@ -11680,7 +11267,7 @@
         <v>129</v>
       </c>
       <c r="J13" s="5" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="K13" s="5" t="s">
         <v>179</v>
@@ -11698,10 +11285,10 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="5" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="C14" s="7"/>
       <c r="D14" s="8"/>
@@ -11719,7 +11306,7 @@
         <v>129</v>
       </c>
       <c r="J14" s="5" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="K14" s="5" t="s">
         <v>179</v>
@@ -11737,10 +11324,10 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="5" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="C15" s="7"/>
       <c r="D15" s="8"/>
@@ -11758,7 +11345,7 @@
         <v>129</v>
       </c>
       <c r="J15" s="5" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="K15" s="5"/>
       <c r="L15" s="5" t="s">
@@ -11774,10 +11361,10 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="5" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="C16" s="7"/>
       <c r="D16" s="8"/>
@@ -11795,7 +11382,7 @@
         <v>129</v>
       </c>
       <c r="J16" s="5" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="K16" s="5"/>
       <c r="L16" s="5" t="s">
@@ -11811,10 +11398,10 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="5" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="C17" s="7"/>
       <c r="D17" s="8"/>
@@ -11832,7 +11419,7 @@
         <v>129</v>
       </c>
       <c r="J17" s="5" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="K17" s="5"/>
       <c r="L17" s="5" t="s">
@@ -11848,10 +11435,10 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="5" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="C18" s="7"/>
       <c r="D18" s="8"/>
@@ -11869,7 +11456,7 @@
         <v>129</v>
       </c>
       <c r="J18" s="5" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="K18" s="5"/>
       <c r="L18" s="5" t="s">
@@ -11885,10 +11472,10 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="5" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="C19" s="7"/>
       <c r="D19" s="8"/>
@@ -11906,7 +11493,7 @@
         <v>131</v>
       </c>
       <c r="J19" s="5" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="K19" s="5" t="s">
         <v>179</v>
@@ -11924,10 +11511,10 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="5" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="C20" s="7"/>
       <c r="D20" s="8"/>
@@ -11963,10 +11550,10 @@
     </row>
     <row r="21" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="5" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="C21" s="7"/>
       <c r="D21" s="8"/>
@@ -11984,7 +11571,7 @@
         <v>131</v>
       </c>
       <c r="J21" s="5" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="K21" s="5" t="s">
         <v>179</v>
@@ -12002,10 +11589,10 @@
     </row>
     <row r="22" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="5" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="C22" s="7"/>
       <c r="D22" s="8"/>
@@ -12023,7 +11610,7 @@
         <v>131</v>
       </c>
       <c r="J22" s="5" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="K22" s="5" t="s">
         <v>179</v>
@@ -12041,10 +11628,10 @@
     </row>
     <row r="23" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="5" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="C23" s="7"/>
       <c r="D23" s="8"/>
@@ -12062,7 +11649,7 @@
         <v>131</v>
       </c>
       <c r="J23" s="5" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="K23" s="5" t="s">
         <v>179</v>
@@ -12080,10 +11667,10 @@
     </row>
     <row r="24" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="5" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="C24" s="7"/>
       <c r="D24" s="8"/>
@@ -12101,7 +11688,7 @@
         <v>131</v>
       </c>
       <c r="J24" s="5" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="K24" s="5" t="s">
         <v>179</v>

</xml_diff>